<commit_message>
Registration window: show retrieved details only when the record gave some; no duplicate notice
Found on test.gokesari.com after #298: the "Retrieved from your GST record" box showed while the
check was only in review (nothing retrieved), and the warning above the document window repeated
the last line's message. Test report and tracker updated with the staging run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/shop-onboarding-wizard-2026-10/SHOP_REGISTRATION_SINGLE_FLOW_TRACKER_2026-10-30.xlsx
+++ b/docs/shop-onboarding-wizard-2026-10/SHOP_REGISTRATION_SINGLE_FLOW_TRACKER_2026-10-30.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="171">
   <si>
     <t>Shop registration — single flow, document window, pin after payment (owner brief 30 Oct 2026)</t>
   </si>
   <si>
-    <t>As of 30 Oct 2026, 23:30 IST. Branch fix/registration-single-flow, PR #298 into staging (CI running). Not on test.gokesari.com or gokesari.com yet. Design: docs/shop-onboarding-wizard-2026-10/FLOW_2026-10-30-b.md.</t>
+    <t>As of 31 Oct 2026, 00:30 IST. PR #298 merged into staging (685e1f2f) and live on test.gokesari.com since 30 Oct 18:37 UTC; follow-up fixes in a second PR. Not on gokesari.com. Design: docs/shop-onboarding-wizard-2026-10/FLOW_2026-10-30-b.md.</t>
   </si>
   <si>
     <t>#</t>
@@ -45,7 +45,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Local; PR #298</t>
+    <t>test.gokesari.com (#298)</t>
   </si>
   <si>
     <t>One card on /sell and Seller Central → /shop/register. /shop/join forwards with ?code=/?ref=. /shop/join/{token} status pages unchanged.</t>
@@ -111,7 +111,7 @@
     <t>Page 4: payment</t>
   </si>
   <si>
-    <t>Unchanged checkout; sandbox payment tested locally.</t>
+    <t>Checkout unchanged. Local: sandbox payment passed. Staging: goes to HDFC Bank UAT gateway — not completed.</t>
   </si>
   <si>
     <t>-</t>
@@ -120,7 +120,10 @@
     <t>Page 5: address and location after payment</t>
   </si>
   <si>
-    <t>Owner chose 'pin after pay': address given before payment (shop needs one), corrected with the map pin after payment.</t>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Owner chose 'pin after pay': address given before payment (shop needs one), corrected with the map pin after payment. Verified locally; not reached on staging because staging's fee payment now goes to HDFC UAT.</t>
   </si>
   <si>
     <t>shop-registration-wizard.ts (step order); onboarding-wizard.tsx (ShopLocationStep)</t>
@@ -129,45 +132,42 @@
     <t>Google Maps fix</t>
   </si>
   <si>
+    <t>test.gokesari.com and gokesari.com</t>
+  </si>
+  <si>
+    <t>Cause: staging was built with a different browser key that Google refused (RefererNotAllowedMapError). Owner set the production key on staging in hPanel; the #298 build carries it and the map loads (verified 30 Oct). Code fallback for a refused key added.</t>
+  </si>
+  <si>
+    <t>lib/geo/provider.ts; map-picker.tsx; nearby-map.tsx</t>
+  </si>
+  <si>
+    <t>Android and iOS apps</t>
+  </si>
+  <si>
+    <t>WebView — no build needed</t>
+  </si>
+  <si>
+    <t>Both apps show the website; changes arrive with the web deploy. No platform differences in this flow.</t>
+  </si>
+  <si>
+    <t>mobile/README.md</t>
+  </si>
+  <si>
+    <t>Testing on Test (test.gokesari.com)</t>
+  </si>
+  <si>
+    <t>After merge of PR #298</t>
+  </si>
+  <si>
+    <t>Steps 1–6 pass on staging. Payment and address/location step blocked: staging uses PAYMENT_GATEWAY=HDFC (UAT), not SANDBOX.</t>
+  </si>
+  <si>
+    <t>Testing on Prod (gokesari.com)</t>
+  </si>
+  <si>
     <t>Blocked</t>
   </si>
   <si>
-    <t>Code fallback in PR #298</t>
-  </si>
-  <si>
-    <t>Cause: staging browser key refused (RefererNotAllowedMapError); production OK. Needs the owner to add https://test.gokesari.com/* to the key's website restrictions in Google Cloud Console. Code fallback added for a refused key.</t>
-  </si>
-  <si>
-    <t>lib/geo/provider.ts; map-picker.tsx; nearby-map.tsx</t>
-  </si>
-  <si>
-    <t>Android and iOS apps</t>
-  </si>
-  <si>
-    <t>WebView — no build needed</t>
-  </si>
-  <si>
-    <t>Both apps show the website; changes arrive with the web deploy. No platform differences in this flow.</t>
-  </si>
-  <si>
-    <t>mobile/README.md</t>
-  </si>
-  <si>
-    <t>Testing on Test (test.gokesari.com)</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>After merge of PR #298</t>
-  </si>
-  <si>
-    <t>Needs: merge into staging, the wizard flag on for staging (Admin → Feature flags), and the Maps key fix.</t>
-  </si>
-  <si>
-    <t>Testing on Prod (gokesari.com)</t>
-  </si>
-  <si>
     <t>Owner-approved release window</t>
   </si>
   <si>
@@ -345,10 +345,34 @@
     <t>Script + Places load, no auth error</t>
   </si>
   <si>
+    <t>REG-1</t>
+  </si>
+  <si>
+    <t>Regression: whole suite</t>
+  </si>
+  <si>
+    <t>see UT-4</t>
+  </si>
+  <si>
+    <t>PRD-1</t>
+  </si>
+  <si>
+    <t>Smoke on gokesari.com</t>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <t>Not run</t>
+  </si>
+  <si>
+    <t>after an owner-approved release</t>
+  </si>
+  <si>
     <t>MAP-2</t>
   </si>
   <si>
-    <t>Maps on test.gokesari.com</t>
+    <t>Maps on test.gokesari.com before the fix</t>
   </si>
   <si>
     <t>Staging</t>
@@ -357,40 +381,91 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>RefererNotAllowedMapError — owner action in Google Cloud Console</t>
-  </si>
-  <si>
-    <t>REG-1</t>
-  </si>
-  <si>
-    <t>Regression: whole suite</t>
-  </si>
-  <si>
-    <t>see UT-4</t>
-  </si>
-  <si>
-    <t>STG-1</t>
-  </si>
-  <si>
-    <t>Registration flow on test.gokesari.com</t>
-  </si>
-  <si>
-    <t>Not run</t>
-  </si>
-  <si>
-    <t>after merge + wizard flag</t>
-  </si>
-  <si>
-    <t>PRD-1</t>
-  </si>
-  <si>
-    <t>Smoke on gokesari.com</t>
-  </si>
-  <si>
-    <t>Production</t>
-  </si>
-  <si>
-    <t>after an owner-approved release</t>
+    <t>RefererNotAllowedMapError with the old staging key</t>
+  </si>
+  <si>
+    <t>MAP-3</t>
+  </si>
+  <si>
+    <t>Maps on test.gokesari.com after the owner's key change</t>
+  </si>
+  <si>
+    <t>Production key (…UffY) built in; map and Places load</t>
+  </si>
+  <si>
+    <t>ST-1</t>
+  </si>
+  <si>
+    <t>/sell one card → /shop/register</t>
+  </si>
+  <si>
+    <t>ST-2</t>
+  </si>
+  <si>
+    <t>/shop/join?code → /shop/register?ref</t>
+  </si>
+  <si>
+    <t>ST-3</t>
+  </si>
+  <si>
+    <t>Seller Central with no shop: one card</t>
+  </si>
+  <si>
+    <t>ST-4</t>
+  </si>
+  <si>
+    <t>Code required on staging; test code T47BC8PU</t>
+  </si>
+  <si>
+    <t>ST-5</t>
+  </si>
+  <si>
+    <t>Referral → email → Yes / No</t>
+  </si>
+  <si>
+    <t>ST-6</t>
+  </si>
+  <si>
+    <t>Document window, 5 lines with Validate</t>
+  </si>
+  <si>
+    <t>Staging provider: all 'Our team will check' for test numbers</t>
+  </si>
+  <si>
+    <t>ST-7</t>
+  </si>
+  <si>
+    <t>Confirm details → review (no map before payment) → shop created</t>
+  </si>
+  <si>
+    <t>QA Staging Stores 298</t>
+  </si>
+  <si>
+    <t>ST-8</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>Goes to HDFC UAT gateway; card details not entered by Claude</t>
+  </si>
+  <si>
+    <t>ST-9</t>
+  </si>
+  <si>
+    <t>Address and location after payment</t>
+  </si>
+  <si>
+    <t>Needs ST-8</t>
+  </si>
+  <si>
+    <t>GOV-STG</t>
+  </si>
+  <si>
+    <t>GSTIN / Shop Act / FSSAI / Udyam on the staging provider</t>
+  </si>
+  <si>
+    <t>Clear 'Our team will check' states; a real GSTIN is needed to see Verified</t>
   </si>
   <si>
     <t>Open items and decisions</t>
@@ -405,7 +480,7 @@
     <t>Who</t>
   </si>
   <si>
-    <t>Add https://test.gokesari.com/* to the staging Maps browser key's website restrictions</t>
+    <t>Production release window</t>
   </si>
   <si>
     <t>Owner</t>
@@ -414,30 +489,6 @@
     <t>Open</t>
   </si>
   <si>
-    <t>Google Cloud Console → Credentials</t>
-  </si>
-  <si>
-    <t>Merge PR #298 into staging after CI</t>
-  </si>
-  <si>
-    <t>Claude / owner</t>
-  </si>
-  <si>
-    <t>Then run STG-1</t>
-  </si>
-  <si>
-    <t>Switch shop_onboarding_wizard_enabled on for test.gokesari.com</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Without it, /shop/register shows the long form to non-admins</t>
-  </si>
-  <si>
-    <t>Production release window</t>
-  </si>
-  <si>
     <t>One release at a time (DEPLOYMENT.md §3)</t>
   </si>
   <si>
@@ -454,6 +505,27 @@
   </si>
   <si>
     <t>Carried from 30 Oct flow</t>
+  </si>
+  <si>
+    <t>Staging fee payment goes to HDFC UAT — switch back to SANDBOX or pay with HDFC's test card</t>
+  </si>
+  <si>
+    <t>Blocks ST-8 / ST-9</t>
+  </si>
+  <si>
+    <t>Dealer-role account sees the wizard but step 1 says 'no permission'</t>
+  </si>
+  <si>
+    <t>Existing; could tell dealers to switch to their customer account</t>
+  </si>
+  <si>
+    <t>Staging test data: shop 'QA Staging Stores 298' (unpaid) and referral code T47BC8PU</t>
+  </si>
+  <si>
+    <t>Owner / QA</t>
+  </si>
+  <si>
+    <t>Delete or keep for the next run</t>
   </si>
 </sst>
 </file>
@@ -499,12 +571,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -1093,17 +1165,17 @@
       <c r="B13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>9</v>
+      <c r="C13" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1111,10 +1183,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="7" t="s">
         <v>38</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>39</v>
@@ -1153,14 +1225,14 @@
       <c r="B16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>33</v>
@@ -1171,10 +1243,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>51</v>
@@ -1194,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1511,27 +1583,27 @@
         <v>111</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="D22" s="9" t="s">
         <v>116</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>117</v>
@@ -1545,30 +1617,200 @@
         <v>119</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="9" t="s">
         <v>120</v>
       </c>
+      <c r="D23" s="8" t="s">
+        <v>121</v>
+      </c>
       <c r="E23" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="9" t="s">
         <v>120</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1591,12 +1833,12 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1604,10 +1846,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>4</v>
@@ -1618,104 +1860,104 @@
     </row>
     <row r="5" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>131</v>
+        <v>169</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>146</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docs: registration single flow — staging run complete (payment and location pass after #299)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/shop-onboarding-wizard-2026-10/SHOP_REGISTRATION_SINGLE_FLOW_TRACKER_2026-10-30.xlsx
+++ b/docs/shop-onboarding-wizard-2026-10/SHOP_REGISTRATION_SINGLE_FLOW_TRACKER_2026-10-30.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="178">
   <si>
     <t>Shop registration — single flow, document window, pin after payment (owner brief 30 Oct 2026)</t>
   </si>
   <si>
-    <t>As of 31 Oct 2026, 00:30 IST. PR #298 merged into staging (685e1f2f) and live on test.gokesari.com since 30 Oct 18:37 UTC; follow-up fixes in a second PR. Not on gokesari.com. Design: docs/shop-onboarding-wizard-2026-10/FLOW_2026-10-30-b.md.</t>
+    <t>As of 31 Oct 2026, 10:00 IST. PR #298 and #299 merged into staging and live on test.gokesari.com; the whole flow passed there on 31 Oct. Not on gokesari.com (waits for an owner-approved release). Design: docs/shop-onboarding-wizard-2026-10/FLOW_2026-10-30-b.md.</t>
   </si>
   <si>
     <t>#</t>
@@ -45,7 +45,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>test.gokesari.com (#298)</t>
+    <t>test.gokesari.com (#298, #299)</t>
   </si>
   <si>
     <t>One card on /sell and Seller Central → /shop/register. /shop/join forwards with ?code=/?ref=. /shop/join/{token} status pages unchanged.</t>
@@ -111,7 +111,7 @@
     <t>Page 4: payment</t>
   </si>
   <si>
-    <t>Checkout unchanged. Local: sandbox payment passed. Staging: goes to HDFC Bank UAT gateway — not completed.</t>
+    <t>Checkout unchanged. Staging (SANDBOX): paid on the built-in sandbox page. Found and fixed a receipt-number bug that stopped payments being recorded (#299).</t>
   </si>
   <si>
     <t>-</t>
@@ -120,10 +120,7 @@
     <t>Page 5: address and location after payment</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Owner chose 'pin after pay': address given before payment (shop needs one), corrected with the map pin after payment. Verified locally; not reached on staging because staging's fee payment now goes to HDFC UAT.</t>
+    <t>Owner chose 'pin after pay'. Staging: after payment and approval, step 8 showed the address pre-filled and the Google map; Confirm location saved address, landmark and pin.</t>
   </si>
   <si>
     <t>shop-registration-wizard.ts (step order); onboarding-wizard.tsx (ShopLocationStep)</t>
@@ -159,7 +156,7 @@
     <t>After merge of PR #298</t>
   </si>
   <si>
-    <t>Steps 1–6 pass on staging. Payment and address/location step blocked: staging uses PAYMENT_GATEWAY=HDFC (UAT), not SANDBOX.</t>
+    <t>Whole flow passed on staging (31 Oct): one card, screen 2, Yes/No, window with Validate, confirm, sandbox payment, address and map location.</t>
   </si>
   <si>
     <t>Testing on Prod (gokesari.com)</t>
@@ -174,6 +171,18 @@
     <t>Owner chose 'staging now, Prod later'. Read-only smoke checks after release; no payment on production.</t>
   </si>
   <si>
+    <t>Payment receipt number fix (found during testing)</t>
+  </si>
+  <si>
+    <t>test.gokesari.com (#299)</t>
+  </si>
+  <si>
+    <t>Receipt = highest number this year + 1 (was row count + 1, which collided after rows were deleted). Must go to production with the next release.</t>
+  </si>
+  <si>
+    <t>src/server/services/shop-payments.ts; tests/integration/shop-payment-reference.test.ts</t>
+  </si>
+  <si>
     <t>Test results</t>
   </si>
   <si>
@@ -447,7 +456,7 @@
     <t>Payment</t>
   </si>
   <si>
-    <t>Goes to HDFC UAT gateway; card details not entered by Claude</t>
+    <t>Sandbox page; captured; recorded after #299 (fee PAID)</t>
   </si>
   <si>
     <t>ST-9</t>
@@ -456,7 +465,7 @@
     <t>Address and location after payment</t>
   </si>
   <si>
-    <t>Needs ST-8</t>
+    <t>Address pre-filled, Google map, Confirm location saved address + landmark + pin (18.5167, 73.8415)</t>
   </si>
   <si>
     <t>GOV-STG</t>
@@ -468,6 +477,18 @@
     <t>Clear 'Our team will check' states; a real GSTIN is needed to see Verified</t>
   </si>
   <si>
+    <t>UT-5</t>
+  </si>
+  <si>
+    <t>Receipt numbers: gap after deleted rows; new year starts at 1</t>
+  </si>
+  <si>
+    <t>Local, both layouts</t>
+  </si>
+  <si>
+    <t>shop-payment-reference.test.ts + payment tests 55 / 55 each</t>
+  </si>
+  <si>
     <t>Open items and decisions</t>
   </si>
   <si>
@@ -507,12 +528,6 @@
     <t>Carried from 30 Oct flow</t>
   </si>
   <si>
-    <t>Staging fee payment goes to HDFC UAT — switch back to SANDBOX or pay with HDFC's test card</t>
-  </si>
-  <si>
-    <t>Blocks ST-8 / ST-9</t>
-  </si>
-  <si>
     <t>Dealer-role account sees the wizard but step 1 says 'no permission'</t>
   </si>
   <si>
@@ -525,7 +540,13 @@
     <t>Owner / QA</t>
   </si>
   <si>
-    <t>Delete or keep for the next run</t>
+    <t>Shops 'QA Staging Stores 298' (unpaid) and 'QA Staging Full Run 298' (live, QA waiver); code T47BC8PU (2 of 5 uses). Delete or keep.</t>
+  </si>
+  <si>
+    <t>Release #298 + #299 to gokesari.com (receipt fix protects production payments)</t>
+  </si>
+  <si>
+    <t>One release at a time; post-deploy check after (DEPLOYMENT.md §3)</t>
   </si>
 </sst>
 </file>
@@ -552,7 +573,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -567,11 +588,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -597,7 +613,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -613,9 +629,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -957,7 +970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1165,17 +1178,17 @@
       <c r="B13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>35</v>
+      <c r="C13" s="6" t="s">
+        <v>9</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1183,19 +1196,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1203,19 +1216,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1223,16 +1236,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>48</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>33</v>
@@ -1243,19 +1256,39 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="D17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1266,7 +1299,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1278,145 +1311,145 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>33</v>
@@ -1424,16 +1457,16 @@
     </row>
     <row r="12" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>33</v>
@@ -1441,84 +1474,84 @@
     </row>
     <row r="13" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>33</v>
@@ -1526,135 +1559,135 @@
     </row>
     <row r="18" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>119</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>124</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>120</v>
-      </c>
       <c r="D24" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>33</v>
@@ -1662,16 +1695,16 @@
     </row>
     <row r="26" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>33</v>
@@ -1679,16 +1712,16 @@
     </row>
     <row r="27" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>33</v>
@@ -1696,33 +1729,33 @@
     </row>
     <row r="28" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>33</v>
@@ -1730,87 +1763,104 @@
     </row>
     <row r="30" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1833,12 +1883,12 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1846,10 +1896,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>4</v>
@@ -1863,16 +1913,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1880,16 +1930,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -1897,67 +1947,67 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>157</v>
-      </c>
       <c r="E8" s="5" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>